<commit_message>
Actualizacion de datos de nueva carpeta
</commit_message>
<xml_diff>
--- a/Animal desconocido 2026/ANIMAL DESCONOCIDO.xlsx
+++ b/Animal desconocido 2026/ANIMAL DESCONOCIDO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\2026\app VACUNACION ANTIRRAVICA 2025 - 2026\Animal desconocido 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7B6B4D-737E-479E-B4E9-B30D8D569758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9246D198-C752-4509-8423-A8F87886D6DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="119">
   <si>
     <t>FUNCIONARIO</t>
   </si>
@@ -271,6 +271,120 @@
   </si>
   <si>
     <t>1.196991, -76.909065</t>
+  </si>
+  <si>
+    <t>bee2b233</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>ALFONZO LOPEZ</t>
+  </si>
+  <si>
+    <t>Esquina de la bomba que está cerca al sementerio</t>
+  </si>
+  <si>
+    <t>Tamaño mediano, semi peludo</t>
+  </si>
+  <si>
+    <t>Negro cafe</t>
+  </si>
+  <si>
+    <t>JOVEN</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/bee2b233.FOTO_ANIMAL.182107.jpg</t>
+  </si>
+  <si>
+    <t>1.152743, -77.002143</t>
+  </si>
+  <si>
+    <t>a2e5f159</t>
+  </si>
+  <si>
+    <t>CRISTO REY</t>
+  </si>
+  <si>
+    <t>Cristo rey</t>
+  </si>
+  <si>
+    <t>GRANDE</t>
+  </si>
+  <si>
+    <t>ENFERMO</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/a2e5f159.FOTO_ANIMAL.135407.jpg</t>
+  </si>
+  <si>
+    <t>TERCERA AGRESION</t>
+  </si>
+  <si>
+    <t>0.663760, -76.863030</t>
+  </si>
+  <si>
+    <t>d680ce12</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Callejón barrio los estudiantes</t>
+  </si>
+  <si>
+    <t>Pelo liso</t>
+  </si>
+  <si>
+    <t>Negro</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/d680ce12.FOTO_ANIMAL.213159.jpg</t>
+  </si>
+  <si>
+    <t>1.147752, -77.003167</t>
+  </si>
+  <si>
+    <t>f620b715</t>
+  </si>
+  <si>
+    <t>VILLA LUISA</t>
+  </si>
+  <si>
+    <t>Calle nueva</t>
+  </si>
+  <si>
+    <t>Mediano</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/f620b715.FOTO_ANIMAL.181618.jpg</t>
+  </si>
+  <si>
+    <t>Su nombre es negra</t>
+  </si>
+  <si>
+    <t>1.147609, -76.997930</t>
+  </si>
+  <si>
+    <t>db9f382d</t>
+  </si>
+  <si>
+    <t>TRIUNFO</t>
+  </si>
+  <si>
+    <t>Última cuadra del barrio el Triunfo</t>
+  </si>
+  <si>
+    <t>Rotwailer y labrador</t>
+  </si>
+  <si>
+    <t>Blanco negro</t>
+  </si>
+  <si>
+    <t>ANIMAL_CALLE_Images/db9f382d.FOTO_ANIMAL.234252.jpg</t>
+  </si>
+  <si>
+    <t>1.147099, -76.997906</t>
   </si>
 </sst>
 </file>
@@ -355,7 +469,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -387,11 +501,25 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -605,7 +733,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" style="2" customWidth="1"/>
@@ -1007,7 +1135,296 @@
         <v>80</v>
       </c>
     </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="10">
+        <v>46273</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="T7" s="5"/>
+      <c r="U7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V7" s="5"/>
+      <c r="W7" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="10">
+        <v>46276</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="T8" s="5"/>
+      <c r="U8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="V8" s="5"/>
+      <c r="W8" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="11">
+        <v>46281</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="T9" s="5"/>
+      <c r="U9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V9" s="5"/>
+      <c r="W9" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="11">
+        <v>46282</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="T10" s="5"/>
+      <c r="U10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="11">
+        <v>46283</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="T11" s="5"/>
+      <c r="V11" s="5"/>
+      <c r="W11" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>